<commit_message>
Use US spelling in scorer workbook and guide
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X72ugjVB4vLu8AESG1BKEi
</commit_message>
<xml_diff>
--- a/prospect-qualification/Fastr_Prospect_Testability_Scorer.xlsx
+++ b/prospect-qualification/Fastr_Prospect_Testability_Scorer.xlsx
@@ -145,7 +145,7 @@
     <t xml:space="preserve">Tier 1 — Pursue</t>
   </si>
   <si>
-    <t xml:space="preserve">A 5% lift reads in ≤ 2 weeks ('Tier 1 (3-wk)' if it takes up to 3). Fast, precise programme. Offer the trial.</t>
+    <t xml:space="preserve">A 5% lift reads in ≤ 2 weeks ('Tier 1 (3-wk)' if it takes up to 3). Fast, precise program. Offer the trial.</t>
   </si>
   <si>
     <t xml:space="preserve">Tier 2 — Qualify</t>
@@ -154,7 +154,7 @@
     <t xml:space="preserve">Only a 10% lift reads within 3 weeks. Bold, funnel-wide tests only. Trial with a scoped plan.</t>
   </si>
   <si>
-    <t xml:space="preserve">Tier 3 — Deprioritise</t>
+    <t xml:space="preserve">Tier 3 — Deprioritize</t>
   </si>
   <si>
     <t xml:space="preserve">Only a 20% lift reads within 3 weeks. Most real wins will be invisible.</t>
@@ -412,7 +412,7 @@
     <t xml:space="preserve">www.jrcigars.com</t>
   </si>
   <si>
-    <t xml:space="preserve">Orders exceed buyers (1.32 per buyer) — repeat buyers. Not previously reviewed: confirm attribution before pitching a programme.</t>
+    <t xml:space="preserve">Orders exceed buyers (1.32 per buyer) — repeat buyers. Not previously reviewed: confirm attribution before pitching a program.</t>
   </si>
   <si>
     <t xml:space="preserve">The Sak</t>
@@ -805,7 +805,7 @@
     <t xml:space="preserve">Maximum acceptable test length (weeks)</t>
   </si>
   <si>
-    <t xml:space="preserve">The brief: 2–3 weeks max. Anything longer is not a fast programme.</t>
+    <t xml:space="preserve">The brief: 2–3 weeks max. Anything longer is not a fast program.</t>
   </si>
   <si>
     <t xml:space="preserve">Lift — typical win (Tier 1 bar)</t>
@@ -2177,8 +2177,8 @@
         <v>Tier 1 (3-wk)</v>
       </c>
       <c r="T5" s="18" t="str">
-        <f aca="false">IF($S5="","",IF(LEFT($S5,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S5="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S5="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S5="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
-        <v>Pursue — trial + fast programme: 5% lifts read in 2–3 weeks</v>
+        <f aca="false">IF($S5="","",IF(LEFT($S5,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S5="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S5="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S5="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <v>Pursue — trial + fast program: 5% lifts read in 2–3 weeks</v>
       </c>
       <c r="U5" s="19" t="n">
         <f aca="false">IF($L5="","",$L5*Assumptions!$C$17*$K5*12/1000000)</f>
@@ -2253,7 +2253,7 @@
         <v>Tier 2</v>
       </c>
       <c r="T6" s="18" t="str">
-        <f aca="false">IF($S6="","",IF(LEFT($S6,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S6="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S6="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S6="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S6="","",IF(LEFT($S6,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S6="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S6="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S6="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v>Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads</v>
       </c>
       <c r="U6" s="19" t="n">
@@ -2327,8 +2327,8 @@
         <v>Tier 1 (3-wk)</v>
       </c>
       <c r="T7" s="18" t="str">
-        <f aca="false">IF($S7="","",IF(LEFT($S7,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S7="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S7="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S7="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
-        <v>Pursue — trial + fast programme: 5% lifts read in 2–3 weeks</v>
+        <f aca="false">IF($S7="","",IF(LEFT($S7,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S7="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S7="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S7="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <v>Pursue — trial + fast program: 5% lifts read in 2–3 weeks</v>
       </c>
       <c r="U7" s="19" t="n">
         <f aca="false">IF($L7="","",$L7*Assumptions!$C$17*$K7*12/1000000)</f>
@@ -2393,7 +2393,7 @@
         <v/>
       </c>
       <c r="T8" s="18" t="str">
-        <f aca="false">IF($S8="","",IF(LEFT($S8,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S8="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S8="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S8="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S8="","",IF(LEFT($S8,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S8="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S8="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S8="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U8" s="19" t="str">
@@ -2459,7 +2459,7 @@
         <v/>
       </c>
       <c r="T9" s="18" t="str">
-        <f aca="false">IF($S9="","",IF(LEFT($S9,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S9="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S9="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S9="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S9="","",IF(LEFT($S9,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S9="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S9="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S9="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U9" s="19" t="str">
@@ -2518,7 +2518,7 @@
         <v/>
       </c>
       <c r="T10" s="18" t="str">
-        <f aca="false">IF($S10="","",IF(LEFT($S10,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S10="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S10="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S10="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S10="","",IF(LEFT($S10,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S10="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S10="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S10="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U10" s="19" t="str">
@@ -2577,7 +2577,7 @@
         <v/>
       </c>
       <c r="T11" s="18" t="str">
-        <f aca="false">IF($S11="","",IF(LEFT($S11,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S11="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S11="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S11="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S11="","",IF(LEFT($S11,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S11="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S11="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S11="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U11" s="19" t="str">
@@ -2636,7 +2636,7 @@
         <v/>
       </c>
       <c r="T12" s="18" t="str">
-        <f aca="false">IF($S12="","",IF(LEFT($S12,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S12="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S12="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S12="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S12="","",IF(LEFT($S12,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S12="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S12="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S12="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U12" s="19" t="str">
@@ -2695,7 +2695,7 @@
         <v/>
       </c>
       <c r="T13" s="18" t="str">
-        <f aca="false">IF($S13="","",IF(LEFT($S13,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S13="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S13="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S13="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S13="","",IF(LEFT($S13,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S13="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S13="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S13="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U13" s="19" t="str">
@@ -2754,7 +2754,7 @@
         <v/>
       </c>
       <c r="T14" s="18" t="str">
-        <f aca="false">IF($S14="","",IF(LEFT($S14,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S14="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S14="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S14="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S14="","",IF(LEFT($S14,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S14="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S14="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S14="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U14" s="19" t="str">
@@ -2813,7 +2813,7 @@
         <v/>
       </c>
       <c r="T15" s="18" t="str">
-        <f aca="false">IF($S15="","",IF(LEFT($S15,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S15="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S15="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S15="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S15="","",IF(LEFT($S15,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S15="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S15="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S15="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U15" s="19" t="str">
@@ -2872,7 +2872,7 @@
         <v/>
       </c>
       <c r="T16" s="18" t="str">
-        <f aca="false">IF($S16="","",IF(LEFT($S16,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S16="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S16="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S16="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S16="","",IF(LEFT($S16,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S16="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S16="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S16="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U16" s="19" t="str">
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
       <c r="T17" s="18" t="str">
-        <f aca="false">IF($S17="","",IF(LEFT($S17,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S17="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S17="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S17="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S17="","",IF(LEFT($S17,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S17="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S17="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S17="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U17" s="19" t="str">
@@ -2990,7 +2990,7 @@
         <v/>
       </c>
       <c r="T18" s="18" t="str">
-        <f aca="false">IF($S18="","",IF(LEFT($S18,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S18="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S18="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S18="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S18="","",IF(LEFT($S18,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S18="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S18="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S18="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U18" s="19" t="str">
@@ -3049,7 +3049,7 @@
         <v/>
       </c>
       <c r="T19" s="18" t="str">
-        <f aca="false">IF($S19="","",IF(LEFT($S19,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S19="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S19="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S19="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S19="","",IF(LEFT($S19,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S19="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S19="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S19="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U19" s="19" t="str">
@@ -3108,7 +3108,7 @@
         <v/>
       </c>
       <c r="T20" s="18" t="str">
-        <f aca="false">IF($S20="","",IF(LEFT($S20,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S20="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S20="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S20="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S20="","",IF(LEFT($S20,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S20="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S20="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S20="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U20" s="19" t="str">
@@ -3167,7 +3167,7 @@
         <v/>
       </c>
       <c r="T21" s="18" t="str">
-        <f aca="false">IF($S21="","",IF(LEFT($S21,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S21="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S21="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S21="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S21="","",IF(LEFT($S21,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S21="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S21="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S21="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U21" s="19" t="str">
@@ -3226,7 +3226,7 @@
         <v/>
       </c>
       <c r="T22" s="18" t="str">
-        <f aca="false">IF($S22="","",IF(LEFT($S22,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S22="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S22="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S22="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S22="","",IF(LEFT($S22,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S22="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S22="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S22="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U22" s="19" t="str">
@@ -3285,7 +3285,7 @@
         <v/>
       </c>
       <c r="T23" s="18" t="str">
-        <f aca="false">IF($S23="","",IF(LEFT($S23,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S23="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S23="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S23="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S23="","",IF(LEFT($S23,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S23="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S23="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S23="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U23" s="19" t="str">
@@ -3344,7 +3344,7 @@
         <v/>
       </c>
       <c r="T24" s="18" t="str">
-        <f aca="false">IF($S24="","",IF(LEFT($S24,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S24="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S24="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S24="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S24="","",IF(LEFT($S24,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S24="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S24="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S24="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U24" s="19" t="str">
@@ -3403,7 +3403,7 @@
         <v/>
       </c>
       <c r="T25" s="18" t="str">
-        <f aca="false">IF($S25="","",IF(LEFT($S25,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S25="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S25="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S25="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S25="","",IF(LEFT($S25,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S25="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S25="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S25="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U25" s="19" t="str">
@@ -3462,7 +3462,7 @@
         <v/>
       </c>
       <c r="T26" s="18" t="str">
-        <f aca="false">IF($S26="","",IF(LEFT($S26,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S26="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S26="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S26="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S26="","",IF(LEFT($S26,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S26="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S26="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S26="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U26" s="19" t="str">
@@ -3521,7 +3521,7 @@
         <v/>
       </c>
       <c r="T27" s="18" t="str">
-        <f aca="false">IF($S27="","",IF(LEFT($S27,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S27="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S27="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S27="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S27="","",IF(LEFT($S27,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S27="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S27="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S27="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U27" s="19" t="str">
@@ -3580,7 +3580,7 @@
         <v/>
       </c>
       <c r="T28" s="18" t="str">
-        <f aca="false">IF($S28="","",IF(LEFT($S28,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S28="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S28="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S28="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S28="","",IF(LEFT($S28,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S28="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S28="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S28="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U28" s="19" t="str">
@@ -3639,7 +3639,7 @@
         <v/>
       </c>
       <c r="T29" s="18" t="str">
-        <f aca="false">IF($S29="","",IF(LEFT($S29,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S29="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S29="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S29="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S29="","",IF(LEFT($S29,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S29="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S29="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S29="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U29" s="19" t="str">
@@ -3698,7 +3698,7 @@
         <v/>
       </c>
       <c r="T30" s="18" t="str">
-        <f aca="false">IF($S30="","",IF(LEFT($S30,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S30="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S30="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S30="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S30="","",IF(LEFT($S30,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S30="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S30="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S30="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U30" s="19" t="str">
@@ -3757,7 +3757,7 @@
         <v/>
       </c>
       <c r="T31" s="18" t="str">
-        <f aca="false">IF($S31="","",IF(LEFT($S31,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S31="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S31="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S31="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S31="","",IF(LEFT($S31,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S31="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S31="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S31="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U31" s="19" t="str">
@@ -3816,7 +3816,7 @@
         <v/>
       </c>
       <c r="T32" s="18" t="str">
-        <f aca="false">IF($S32="","",IF(LEFT($S32,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S32="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S32="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S32="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S32="","",IF(LEFT($S32,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S32="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S32="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S32="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U32" s="19" t="str">
@@ -3875,7 +3875,7 @@
         <v/>
       </c>
       <c r="T33" s="18" t="str">
-        <f aca="false">IF($S33="","",IF(LEFT($S33,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S33="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S33="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S33="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S33="","",IF(LEFT($S33,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S33="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S33="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S33="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U33" s="19" t="str">
@@ -3934,7 +3934,7 @@
         <v/>
       </c>
       <c r="T34" s="18" t="str">
-        <f aca="false">IF($S34="","",IF(LEFT($S34,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S34="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S34="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S34="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S34="","",IF(LEFT($S34,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S34="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S34="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S34="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U34" s="19" t="str">
@@ -3993,7 +3993,7 @@
         <v/>
       </c>
       <c r="T35" s="18" t="str">
-        <f aca="false">IF($S35="","",IF(LEFT($S35,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S35="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S35="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S35="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S35="","",IF(LEFT($S35,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S35="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S35="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S35="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U35" s="19" t="str">
@@ -4052,7 +4052,7 @@
         <v/>
       </c>
       <c r="T36" s="18" t="str">
-        <f aca="false">IF($S36="","",IF(LEFT($S36,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S36="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S36="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S36="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S36="","",IF(LEFT($S36,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S36="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S36="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S36="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U36" s="19" t="str">
@@ -4111,7 +4111,7 @@
         <v/>
       </c>
       <c r="T37" s="18" t="str">
-        <f aca="false">IF($S37="","",IF(LEFT($S37,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S37="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S37="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S37="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S37="","",IF(LEFT($S37,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S37="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S37="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S37="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U37" s="19" t="str">
@@ -4170,7 +4170,7 @@
         <v/>
       </c>
       <c r="T38" s="18" t="str">
-        <f aca="false">IF($S38="","",IF(LEFT($S38,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S38="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S38="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S38="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S38="","",IF(LEFT($S38,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S38="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S38="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S38="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U38" s="19" t="str">
@@ -4229,7 +4229,7 @@
         <v/>
       </c>
       <c r="T39" s="18" t="str">
-        <f aca="false">IF($S39="","",IF(LEFT($S39,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S39="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S39="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S39="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S39="","",IF(LEFT($S39,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S39="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S39="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S39="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U39" s="19" t="str">
@@ -4288,7 +4288,7 @@
         <v/>
       </c>
       <c r="T40" s="18" t="str">
-        <f aca="false">IF($S40="","",IF(LEFT($S40,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S40="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S40="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S40="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S40="","",IF(LEFT($S40,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S40="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S40="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S40="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U40" s="19" t="str">
@@ -4347,7 +4347,7 @@
         <v/>
       </c>
       <c r="T41" s="18" t="str">
-        <f aca="false">IF($S41="","",IF(LEFT($S41,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S41="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S41="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S41="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S41="","",IF(LEFT($S41,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S41="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S41="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S41="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U41" s="19" t="str">
@@ -4406,7 +4406,7 @@
         <v/>
       </c>
       <c r="T42" s="18" t="str">
-        <f aca="false">IF($S42="","",IF(LEFT($S42,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S42="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S42="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S42="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S42="","",IF(LEFT($S42,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S42="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S42="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S42="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U42" s="19" t="str">
@@ -4465,7 +4465,7 @@
         <v/>
       </c>
       <c r="T43" s="18" t="str">
-        <f aca="false">IF($S43="","",IF(LEFT($S43,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S43="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S43="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S43="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S43="","",IF(LEFT($S43,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S43="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S43="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S43="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U43" s="19" t="str">
@@ -4524,7 +4524,7 @@
         <v/>
       </c>
       <c r="T44" s="18" t="str">
-        <f aca="false">IF($S44="","",IF(LEFT($S44,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S44="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S44="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S44="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S44="","",IF(LEFT($S44,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S44="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S44="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S44="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U44" s="19" t="str">
@@ -4583,7 +4583,7 @@
         <v/>
       </c>
       <c r="T45" s="18" t="str">
-        <f aca="false">IF($S45="","",IF(LEFT($S45,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S45="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S45="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S45="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S45="","",IF(LEFT($S45,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S45="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S45="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S45="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U45" s="19" t="str">
@@ -4642,7 +4642,7 @@
         <v/>
       </c>
       <c r="T46" s="18" t="str">
-        <f aca="false">IF($S46="","",IF(LEFT($S46,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S46="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S46="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S46="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S46="","",IF(LEFT($S46,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S46="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S46="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S46="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U46" s="19" t="str">
@@ -4701,7 +4701,7 @@
         <v/>
       </c>
       <c r="T47" s="18" t="str">
-        <f aca="false">IF($S47="","",IF(LEFT($S47,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S47="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S47="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S47="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S47="","",IF(LEFT($S47,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S47="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S47="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S47="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U47" s="19" t="str">
@@ -4760,7 +4760,7 @@
         <v/>
       </c>
       <c r="T48" s="18" t="str">
-        <f aca="false">IF($S48="","",IF(LEFT($S48,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S48="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S48="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S48="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S48="","",IF(LEFT($S48,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S48="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S48="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S48="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U48" s="19" t="str">
@@ -4819,7 +4819,7 @@
         <v/>
       </c>
       <c r="T49" s="18" t="str">
-        <f aca="false">IF($S49="","",IF(LEFT($S49,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S49="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S49="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S49="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S49="","",IF(LEFT($S49,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S49="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S49="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S49="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U49" s="19" t="str">
@@ -4878,7 +4878,7 @@
         <v/>
       </c>
       <c r="T50" s="18" t="str">
-        <f aca="false">IF($S50="","",IF(LEFT($S50,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S50="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S50="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S50="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S50="","",IF(LEFT($S50,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S50="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S50="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S50="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U50" s="19" t="str">
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="T51" s="18" t="str">
-        <f aca="false">IF($S51="","",IF(LEFT($S51,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S51="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S51="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S51="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S51="","",IF(LEFT($S51,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S51="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S51="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S51="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U51" s="19" t="str">
@@ -4996,7 +4996,7 @@
         <v/>
       </c>
       <c r="T52" s="18" t="str">
-        <f aca="false">IF($S52="","",IF(LEFT($S52,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S52="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S52="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S52="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S52="","",IF(LEFT($S52,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S52="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S52="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S52="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U52" s="19" t="str">
@@ -5055,7 +5055,7 @@
         <v/>
       </c>
       <c r="T53" s="18" t="str">
-        <f aca="false">IF($S53="","",IF(LEFT($S53,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S53="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S53="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S53="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S53="","",IF(LEFT($S53,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S53="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S53="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S53="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U53" s="19" t="str">
@@ -5114,7 +5114,7 @@
         <v/>
       </c>
       <c r="T54" s="18" t="str">
-        <f aca="false">IF($S54="","",IF(LEFT($S54,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S54="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S54="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S54="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S54="","",IF(LEFT($S54,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S54="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S54="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S54="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U54" s="19" t="str">
@@ -5173,7 +5173,7 @@
         <v/>
       </c>
       <c r="T55" s="18" t="str">
-        <f aca="false">IF($S55="","",IF(LEFT($S55,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S55="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S55="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S55="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S55="","",IF(LEFT($S55,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S55="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S55="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S55="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U55" s="19" t="str">
@@ -5232,7 +5232,7 @@
         <v/>
       </c>
       <c r="T56" s="18" t="str">
-        <f aca="false">IF($S56="","",IF(LEFT($S56,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S56="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S56="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S56="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S56="","",IF(LEFT($S56,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S56="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S56="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S56="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U56" s="19" t="str">
@@ -5291,7 +5291,7 @@
         <v/>
       </c>
       <c r="T57" s="18" t="str">
-        <f aca="false">IF($S57="","",IF(LEFT($S57,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S57="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S57="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S57="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S57="","",IF(LEFT($S57,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S57="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S57="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S57="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U57" s="19" t="str">
@@ -5350,7 +5350,7 @@
         <v/>
       </c>
       <c r="T58" s="18" t="str">
-        <f aca="false">IF($S58="","",IF(LEFT($S58,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S58="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S58="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S58="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S58="","",IF(LEFT($S58,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S58="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S58="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S58="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U58" s="19" t="str">
@@ -5409,7 +5409,7 @@
         <v/>
       </c>
       <c r="T59" s="18" t="str">
-        <f aca="false">IF($S59="","",IF(LEFT($S59,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S59="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S59="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S59="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S59="","",IF(LEFT($S59,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S59="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S59="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S59="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U59" s="19" t="str">
@@ -5468,7 +5468,7 @@
         <v/>
       </c>
       <c r="T60" s="18" t="str">
-        <f aca="false">IF($S60="","",IF(LEFT($S60,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S60="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S60="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S60="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S60="","",IF(LEFT($S60,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S60="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S60="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S60="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U60" s="19" t="str">
@@ -5527,7 +5527,7 @@
         <v/>
       </c>
       <c r="T61" s="18" t="str">
-        <f aca="false">IF($S61="","",IF(LEFT($S61,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S61="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S61="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S61="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S61="","",IF(LEFT($S61,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S61="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S61="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S61="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U61" s="19" t="str">
@@ -5586,7 +5586,7 @@
         <v/>
       </c>
       <c r="T62" s="18" t="str">
-        <f aca="false">IF($S62="","",IF(LEFT($S62,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S62="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S62="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S62="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S62="","",IF(LEFT($S62,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S62="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S62="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S62="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U62" s="19" t="str">
@@ -5645,7 +5645,7 @@
         <v/>
       </c>
       <c r="T63" s="18" t="str">
-        <f aca="false">IF($S63="","",IF(LEFT($S63,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S63="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S63="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S63="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S63="","",IF(LEFT($S63,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S63="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S63="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S63="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U63" s="19" t="str">
@@ -5704,7 +5704,7 @@
         <v/>
       </c>
       <c r="T64" s="18" t="str">
-        <f aca="false">IF($S64="","",IF(LEFT($S64,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S64="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S64="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S64="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S64="","",IF(LEFT($S64,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S64="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S64="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S64="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U64" s="19" t="str">
@@ -5763,7 +5763,7 @@
         <v/>
       </c>
       <c r="T65" s="18" t="str">
-        <f aca="false">IF($S65="","",IF(LEFT($S65,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S65="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S65="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S65="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S65="","",IF(LEFT($S65,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S65="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S65="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S65="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U65" s="19" t="str">
@@ -5822,7 +5822,7 @@
         <v/>
       </c>
       <c r="T66" s="18" t="str">
-        <f aca="false">IF($S66="","",IF(LEFT($S66,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S66="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S66="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S66="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S66="","",IF(LEFT($S66,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S66="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S66="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S66="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U66" s="19" t="str">
@@ -5881,7 +5881,7 @@
         <v/>
       </c>
       <c r="T67" s="18" t="str">
-        <f aca="false">IF($S67="","",IF(LEFT($S67,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S67="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S67="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S67="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S67="","",IF(LEFT($S67,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S67="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S67="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S67="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U67" s="19" t="str">
@@ -5940,7 +5940,7 @@
         <v/>
       </c>
       <c r="T68" s="18" t="str">
-        <f aca="false">IF($S68="","",IF(LEFT($S68,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S68="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S68="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S68="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S68="","",IF(LEFT($S68,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S68="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S68="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S68="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U68" s="19" t="str">
@@ -5999,7 +5999,7 @@
         <v/>
       </c>
       <c r="T69" s="18" t="str">
-        <f aca="false">IF($S69="","",IF(LEFT($S69,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S69="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S69="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S69="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S69="","",IF(LEFT($S69,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S69="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S69="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S69="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U69" s="19" t="str">
@@ -6058,7 +6058,7 @@
         <v/>
       </c>
       <c r="T70" s="18" t="str">
-        <f aca="false">IF($S70="","",IF(LEFT($S70,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S70="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S70="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S70="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S70="","",IF(LEFT($S70,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S70="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S70="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S70="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U70" s="19" t="str">
@@ -6117,7 +6117,7 @@
         <v/>
       </c>
       <c r="T71" s="18" t="str">
-        <f aca="false">IF($S71="","",IF(LEFT($S71,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S71="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S71="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S71="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S71="","",IF(LEFT($S71,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S71="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S71="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S71="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U71" s="19" t="str">
@@ -6176,7 +6176,7 @@
         <v/>
       </c>
       <c r="T72" s="18" t="str">
-        <f aca="false">IF($S72="","",IF(LEFT($S72,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S72="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S72="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S72="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S72="","",IF(LEFT($S72,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S72="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S72="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S72="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U72" s="19" t="str">
@@ -6235,7 +6235,7 @@
         <v/>
       </c>
       <c r="T73" s="18" t="str">
-        <f aca="false">IF($S73="","",IF(LEFT($S73,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S73="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S73="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S73="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S73="","",IF(LEFT($S73,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S73="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S73="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S73="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U73" s="19" t="str">
@@ -6294,7 +6294,7 @@
         <v/>
       </c>
       <c r="T74" s="18" t="str">
-        <f aca="false">IF($S74="","",IF(LEFT($S74,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S74="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S74="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S74="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S74="","",IF(LEFT($S74,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S74="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S74="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S74="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U74" s="19" t="str">
@@ -6353,7 +6353,7 @@
         <v/>
       </c>
       <c r="T75" s="18" t="str">
-        <f aca="false">IF($S75="","",IF(LEFT($S75,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S75="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S75="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S75="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S75="","",IF(LEFT($S75,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S75="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S75="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S75="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U75" s="19" t="str">
@@ -6412,7 +6412,7 @@
         <v/>
       </c>
       <c r="T76" s="18" t="str">
-        <f aca="false">IF($S76="","",IF(LEFT($S76,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S76="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S76="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S76="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S76="","",IF(LEFT($S76,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S76="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S76="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S76="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U76" s="19" t="str">
@@ -6471,7 +6471,7 @@
         <v/>
       </c>
       <c r="T77" s="18" t="str">
-        <f aca="false">IF($S77="","",IF(LEFT($S77,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S77="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S77="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S77="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S77="","",IF(LEFT($S77,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S77="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S77="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S77="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U77" s="19" t="str">
@@ -6530,7 +6530,7 @@
         <v/>
       </c>
       <c r="T78" s="18" t="str">
-        <f aca="false">IF($S78="","",IF(LEFT($S78,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S78="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S78="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S78="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S78="","",IF(LEFT($S78,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S78="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S78="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S78="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U78" s="19" t="str">
@@ -6589,7 +6589,7 @@
         <v/>
       </c>
       <c r="T79" s="18" t="str">
-        <f aca="false">IF($S79="","",IF(LEFT($S79,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S79="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S79="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S79="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S79="","",IF(LEFT($S79,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S79="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S79="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S79="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U79" s="19" t="str">
@@ -6648,7 +6648,7 @@
         <v/>
       </c>
       <c r="T80" s="18" t="str">
-        <f aca="false">IF($S80="","",IF(LEFT($S80,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S80="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S80="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S80="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S80="","",IF(LEFT($S80,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S80="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S80="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S80="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U80" s="19" t="str">
@@ -6707,7 +6707,7 @@
         <v/>
       </c>
       <c r="T81" s="18" t="str">
-        <f aca="false">IF($S81="","",IF(LEFT($S81,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S81="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S81="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S81="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S81="","",IF(LEFT($S81,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S81="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S81="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S81="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U81" s="19" t="str">
@@ -6766,7 +6766,7 @@
         <v/>
       </c>
       <c r="T82" s="18" t="str">
-        <f aca="false">IF($S82="","",IF(LEFT($S82,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S82="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S82="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S82="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S82="","",IF(LEFT($S82,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S82="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S82="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S82="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U82" s="19" t="str">
@@ -6825,7 +6825,7 @@
         <v/>
       </c>
       <c r="T83" s="18" t="str">
-        <f aca="false">IF($S83="","",IF(LEFT($S83,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S83="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S83="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S83="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S83="","",IF(LEFT($S83,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S83="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S83="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S83="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U83" s="19" t="str">
@@ -6884,7 +6884,7 @@
         <v/>
       </c>
       <c r="T84" s="18" t="str">
-        <f aca="false">IF($S84="","",IF(LEFT($S84,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S84="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S84="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S84="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S84="","",IF(LEFT($S84,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S84="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S84="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S84="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U84" s="19" t="str">
@@ -6943,7 +6943,7 @@
         <v/>
       </c>
       <c r="T85" s="18" t="str">
-        <f aca="false">IF($S85="","",IF(LEFT($S85,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S85="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S85="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S85="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S85="","",IF(LEFT($S85,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S85="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S85="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S85="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U85" s="19" t="str">
@@ -7002,7 +7002,7 @@
         <v/>
       </c>
       <c r="T86" s="18" t="str">
-        <f aca="false">IF($S86="","",IF(LEFT($S86,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S86="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S86="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S86="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S86="","",IF(LEFT($S86,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S86="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S86="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S86="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U86" s="19" t="str">
@@ -7061,7 +7061,7 @@
         <v/>
       </c>
       <c r="T87" s="18" t="str">
-        <f aca="false">IF($S87="","",IF(LEFT($S87,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S87="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S87="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S87="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S87="","",IF(LEFT($S87,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S87="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S87="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S87="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U87" s="19" t="str">
@@ -7120,7 +7120,7 @@
         <v/>
       </c>
       <c r="T88" s="18" t="str">
-        <f aca="false">IF($S88="","",IF(LEFT($S88,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S88="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S88="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S88="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S88="","",IF(LEFT($S88,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S88="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S88="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S88="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U88" s="19" t="str">
@@ -7179,7 +7179,7 @@
         <v/>
       </c>
       <c r="T89" s="18" t="str">
-        <f aca="false">IF($S89="","",IF(LEFT($S89,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S89="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S89="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S89="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S89="","",IF(LEFT($S89,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S89="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S89="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S89="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U89" s="19" t="str">
@@ -7238,7 +7238,7 @@
         <v/>
       </c>
       <c r="T90" s="18" t="str">
-        <f aca="false">IF($S90="","",IF(LEFT($S90,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S90="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S90="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S90="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S90="","",IF(LEFT($S90,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S90="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S90="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S90="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U90" s="19" t="str">
@@ -7297,7 +7297,7 @@
         <v/>
       </c>
       <c r="T91" s="18" t="str">
-        <f aca="false">IF($S91="","",IF(LEFT($S91,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S91="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S91="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S91="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S91="","",IF(LEFT($S91,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S91="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S91="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S91="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U91" s="19" t="str">
@@ -7356,7 +7356,7 @@
         <v/>
       </c>
       <c r="T92" s="18" t="str">
-        <f aca="false">IF($S92="","",IF(LEFT($S92,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S92="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S92="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S92="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S92="","",IF(LEFT($S92,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S92="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S92="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S92="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U92" s="19" t="str">
@@ -7415,7 +7415,7 @@
         <v/>
       </c>
       <c r="T93" s="18" t="str">
-        <f aca="false">IF($S93="","",IF(LEFT($S93,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S93="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S93="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S93="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S93="","",IF(LEFT($S93,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S93="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S93="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S93="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U93" s="19" t="str">
@@ -7474,7 +7474,7 @@
         <v/>
       </c>
       <c r="T94" s="18" t="str">
-        <f aca="false">IF($S94="","",IF(LEFT($S94,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S94="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S94="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S94="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S94="","",IF(LEFT($S94,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S94="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S94="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S94="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U94" s="19" t="str">
@@ -7533,7 +7533,7 @@
         <v/>
       </c>
       <c r="T95" s="18" t="str">
-        <f aca="false">IF($S95="","",IF(LEFT($S95,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S95="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S95="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S95="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S95="","",IF(LEFT($S95,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S95="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S95="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S95="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U95" s="19" t="str">
@@ -7592,7 +7592,7 @@
         <v/>
       </c>
       <c r="T96" s="18" t="str">
-        <f aca="false">IF($S96="","",IF(LEFT($S96,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S96="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S96="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S96="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S96="","",IF(LEFT($S96,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S96="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S96="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S96="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U96" s="19" t="str">
@@ -7651,7 +7651,7 @@
         <v/>
       </c>
       <c r="T97" s="18" t="str">
-        <f aca="false">IF($S97="","",IF(LEFT($S97,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S97="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S97="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S97="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S97="","",IF(LEFT($S97,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S97="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S97="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S97="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U97" s="19" t="str">
@@ -7710,7 +7710,7 @@
         <v/>
       </c>
       <c r="T98" s="18" t="str">
-        <f aca="false">IF($S98="","",IF(LEFT($S98,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S98="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S98="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S98="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S98="","",IF(LEFT($S98,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S98="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S98="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S98="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U98" s="19" t="str">
@@ -7769,7 +7769,7 @@
         <v/>
       </c>
       <c r="T99" s="18" t="str">
-        <f aca="false">IF($S99="","",IF(LEFT($S99,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S99="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S99="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S99="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S99="","",IF(LEFT($S99,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S99="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S99="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S99="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U99" s="19" t="str">
@@ -7828,7 +7828,7 @@
         <v/>
       </c>
       <c r="T100" s="18" t="str">
-        <f aca="false">IF($S100="","",IF(LEFT($S100,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S100="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S100="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S100="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S100="","",IF(LEFT($S100,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S100="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S100="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S100="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U100" s="19" t="str">
@@ -7887,7 +7887,7 @@
         <v/>
       </c>
       <c r="T101" s="18" t="str">
-        <f aca="false">IF($S101="","",IF(LEFT($S101,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S101="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S101="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S101="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S101="","",IF(LEFT($S101,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S101="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S101="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S101="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U101" s="19" t="str">
@@ -7946,7 +7946,7 @@
         <v/>
       </c>
       <c r="T102" s="18" t="str">
-        <f aca="false">IF($S102="","",IF(LEFT($S102,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S102="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S102="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S102="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S102="","",IF(LEFT($S102,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S102="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S102="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S102="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U102" s="19" t="str">
@@ -8005,7 +8005,7 @@
         <v/>
       </c>
       <c r="T103" s="18" t="str">
-        <f aca="false">IF($S103="","",IF(LEFT($S103,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S103="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S103="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S103="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S103="","",IF(LEFT($S103,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S103="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S103="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S103="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U103" s="19" t="str">
@@ -8064,7 +8064,7 @@
         <v/>
       </c>
       <c r="T104" s="18" t="str">
-        <f aca="false">IF($S104="","",IF(LEFT($S104,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S104="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S104="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S104="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S104="","",IF(LEFT($S104,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S104="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S104="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S104="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U104" s="19" t="str">
@@ -8123,7 +8123,7 @@
         <v/>
       </c>
       <c r="T105" s="18" t="str">
-        <f aca="false">IF($S105="","",IF(LEFT($S105,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S105="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S105="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S105="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S105="","",IF(LEFT($S105,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S105="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S105="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S105="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U105" s="19" t="str">
@@ -8182,7 +8182,7 @@
         <v/>
       </c>
       <c r="T106" s="18" t="str">
-        <f aca="false">IF($S106="","",IF(LEFT($S106,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S106="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S106="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S106="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S106="","",IF(LEFT($S106,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S106="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S106="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S106="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U106" s="19" t="str">
@@ -8241,7 +8241,7 @@
         <v/>
       </c>
       <c r="T107" s="18" t="str">
-        <f aca="false">IF($S107="","",IF(LEFT($S107,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S107="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S107="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S107="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S107="","",IF(LEFT($S107,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S107="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S107="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S107="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U107" s="19" t="str">
@@ -8300,7 +8300,7 @@
         <v/>
       </c>
       <c r="T108" s="18" t="str">
-        <f aca="false">IF($S108="","",IF(LEFT($S108,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S108="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S108="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S108="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S108="","",IF(LEFT($S108,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S108="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S108="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S108="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U108" s="19" t="str">
@@ -8359,7 +8359,7 @@
         <v/>
       </c>
       <c r="T109" s="18" t="str">
-        <f aca="false">IF($S109="","",IF(LEFT($S109,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S109="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S109="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S109="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S109="","",IF(LEFT($S109,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S109="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S109="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S109="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U109" s="19" t="str">
@@ -8418,7 +8418,7 @@
         <v/>
       </c>
       <c r="T110" s="18" t="str">
-        <f aca="false">IF($S110="","",IF(LEFT($S110,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S110="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S110="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S110="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S110="","",IF(LEFT($S110,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S110="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S110="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S110="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U110" s="19" t="str">
@@ -8477,7 +8477,7 @@
         <v/>
       </c>
       <c r="T111" s="18" t="str">
-        <f aca="false">IF($S111="","",IF(LEFT($S111,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S111="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S111="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S111="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S111="","",IF(LEFT($S111,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S111="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S111="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S111="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U111" s="19" t="str">
@@ -8536,7 +8536,7 @@
         <v/>
       </c>
       <c r="T112" s="18" t="str">
-        <f aca="false">IF($S112="","",IF(LEFT($S112,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S112="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S112="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S112="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S112="","",IF(LEFT($S112,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S112="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S112="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S112="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U112" s="19" t="str">
@@ -8595,7 +8595,7 @@
         <v/>
       </c>
       <c r="T113" s="18" t="str">
-        <f aca="false">IF($S113="","",IF(LEFT($S113,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S113="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S113="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S113="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S113="","",IF(LEFT($S113,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S113="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S113="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S113="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U113" s="19" t="str">
@@ -8654,7 +8654,7 @@
         <v/>
       </c>
       <c r="T114" s="18" t="str">
-        <f aca="false">IF($S114="","",IF(LEFT($S114,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S114="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S114="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S114="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S114="","",IF(LEFT($S114,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S114="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S114="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S114="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U114" s="19" t="str">
@@ -8713,7 +8713,7 @@
         <v/>
       </c>
       <c r="T115" s="18" t="str">
-        <f aca="false">IF($S115="","",IF(LEFT($S115,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S115="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S115="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S115="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S115="","",IF(LEFT($S115,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S115="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S115="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S115="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U115" s="19" t="str">
@@ -8772,7 +8772,7 @@
         <v/>
       </c>
       <c r="T116" s="18" t="str">
-        <f aca="false">IF($S116="","",IF(LEFT($S116,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S116="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S116="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S116="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S116="","",IF(LEFT($S116,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S116="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S116="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S116="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U116" s="19" t="str">
@@ -8831,7 +8831,7 @@
         <v/>
       </c>
       <c r="T117" s="18" t="str">
-        <f aca="false">IF($S117="","",IF(LEFT($S117,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S117="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S117="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S117="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S117="","",IF(LEFT($S117,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S117="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S117="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S117="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U117" s="19" t="str">
@@ -8890,7 +8890,7 @@
         <v/>
       </c>
       <c r="T118" s="18" t="str">
-        <f aca="false">IF($S118="","",IF(LEFT($S118,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S118="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S118="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S118="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S118="","",IF(LEFT($S118,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S118="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S118="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S118="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U118" s="19" t="str">
@@ -8949,7 +8949,7 @@
         <v/>
       </c>
       <c r="T119" s="18" t="str">
-        <f aca="false">IF($S119="","",IF(LEFT($S119,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S119="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S119="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S119="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S119="","",IF(LEFT($S119,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S119="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S119="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S119="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U119" s="19" t="str">
@@ -9008,7 +9008,7 @@
         <v/>
       </c>
       <c r="T120" s="18" t="str">
-        <f aca="false">IF($S120="","",IF(LEFT($S120,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S120="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S120="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S120="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S120="","",IF(LEFT($S120,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S120="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S120="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S120="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U120" s="19" t="str">
@@ -9067,7 +9067,7 @@
         <v/>
       </c>
       <c r="T121" s="18" t="str">
-        <f aca="false">IF($S121="","",IF(LEFT($S121,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S121="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S121="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S121="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S121="","",IF(LEFT($S121,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S121="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S121="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S121="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U121" s="19" t="str">
@@ -9126,7 +9126,7 @@
         <v/>
       </c>
       <c r="T122" s="18" t="str">
-        <f aca="false">IF($S122="","",IF(LEFT($S122,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S122="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S122="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S122="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S122="","",IF(LEFT($S122,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S122="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S122="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S122="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U122" s="19" t="str">
@@ -9185,7 +9185,7 @@
         <v/>
       </c>
       <c r="T123" s="18" t="str">
-        <f aca="false">IF($S123="","",IF(LEFT($S123,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S123="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S123="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S123="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S123="","",IF(LEFT($S123,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S123="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S123="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S123="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U123" s="19" t="str">
@@ -9244,7 +9244,7 @@
         <v/>
       </c>
       <c r="T124" s="18" t="str">
-        <f aca="false">IF($S124="","",IF(LEFT($S124,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S124="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S124="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S124="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S124="","",IF(LEFT($S124,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S124="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S124="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S124="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U124" s="19" t="str">
@@ -9303,7 +9303,7 @@
         <v/>
       </c>
       <c r="T125" s="18" t="str">
-        <f aca="false">IF($S125="","",IF(LEFT($S125,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S125="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S125="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S125="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S125="","",IF(LEFT($S125,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S125="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S125="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S125="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U125" s="19" t="str">
@@ -9362,7 +9362,7 @@
         <v/>
       </c>
       <c r="T126" s="18" t="str">
-        <f aca="false">IF($S126="","",IF(LEFT($S126,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S126="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S126="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S126="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S126="","",IF(LEFT($S126,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S126="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S126="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S126="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U126" s="19" t="str">
@@ -9421,7 +9421,7 @@
         <v/>
       </c>
       <c r="T127" s="18" t="str">
-        <f aca="false">IF($S127="","",IF(LEFT($S127,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S127="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S127="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S127="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S127="","",IF(LEFT($S127,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S127="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S127="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S127="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U127" s="19" t="str">
@@ -9480,7 +9480,7 @@
         <v/>
       </c>
       <c r="T128" s="18" t="str">
-        <f aca="false">IF($S128="","",IF(LEFT($S128,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S128="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S128="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S128="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S128="","",IF(LEFT($S128,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S128="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S128="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S128="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U128" s="19" t="str">
@@ -9539,7 +9539,7 @@
         <v/>
       </c>
       <c r="T129" s="18" t="str">
-        <f aca="false">IF($S129="","",IF(LEFT($S129,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S129="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S129="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S129="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S129="","",IF(LEFT($S129,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S129="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S129="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S129="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U129" s="19" t="str">
@@ -9598,7 +9598,7 @@
         <v/>
       </c>
       <c r="T130" s="18" t="str">
-        <f aca="false">IF($S130="","",IF(LEFT($S130,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S130="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S130="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S130="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S130="","",IF(LEFT($S130,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S130="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S130="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S130="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U130" s="19" t="str">
@@ -9657,7 +9657,7 @@
         <v/>
       </c>
       <c r="T131" s="18" t="str">
-        <f aca="false">IF($S131="","",IF(LEFT($S131,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S131="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S131="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S131="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S131="","",IF(LEFT($S131,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S131="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S131="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S131="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U131" s="19" t="str">
@@ -9716,7 +9716,7 @@
         <v/>
       </c>
       <c r="T132" s="18" t="str">
-        <f aca="false">IF($S132="","",IF(LEFT($S132,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S132="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S132="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S132="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S132="","",IF(LEFT($S132,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S132="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S132="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S132="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U132" s="19" t="str">
@@ -9775,7 +9775,7 @@
         <v/>
       </c>
       <c r="T133" s="18" t="str">
-        <f aca="false">IF($S133="","",IF(LEFT($S133,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S133="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S133="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S133="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S133="","",IF(LEFT($S133,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S133="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S133="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S133="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U133" s="19" t="str">
@@ -9834,7 +9834,7 @@
         <v/>
       </c>
       <c r="T134" s="18" t="str">
-        <f aca="false">IF($S134="","",IF(LEFT($S134,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S134="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S134="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S134="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S134="","",IF(LEFT($S134,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S134="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S134="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S134="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U134" s="19" t="str">
@@ -9893,7 +9893,7 @@
         <v/>
       </c>
       <c r="T135" s="18" t="str">
-        <f aca="false">IF($S135="","",IF(LEFT($S135,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S135="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S135="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S135="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S135="","",IF(LEFT($S135,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S135="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S135="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S135="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U135" s="19" t="str">
@@ -9952,7 +9952,7 @@
         <v/>
       </c>
       <c r="T136" s="18" t="str">
-        <f aca="false">IF($S136="","",IF(LEFT($S136,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S136="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S136="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S136="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S136="","",IF(LEFT($S136,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S136="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S136="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S136="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U136" s="19" t="str">
@@ -10011,7 +10011,7 @@
         <v/>
       </c>
       <c r="T137" s="18" t="str">
-        <f aca="false">IF($S137="","",IF(LEFT($S137,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S137="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S137="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S137="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S137="","",IF(LEFT($S137,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S137="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S137="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S137="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U137" s="19" t="str">
@@ -10070,7 +10070,7 @@
         <v/>
       </c>
       <c r="T138" s="18" t="str">
-        <f aca="false">IF($S138="","",IF(LEFT($S138,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S138="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S138="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S138="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S138="","",IF(LEFT($S138,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S138="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S138="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S138="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U138" s="19" t="str">
@@ -10129,7 +10129,7 @@
         <v/>
       </c>
       <c r="T139" s="18" t="str">
-        <f aca="false">IF($S139="","",IF(LEFT($S139,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S139="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S139="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S139="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S139="","",IF(LEFT($S139,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S139="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S139="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S139="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U139" s="19" t="str">
@@ -10188,7 +10188,7 @@
         <v/>
       </c>
       <c r="T140" s="18" t="str">
-        <f aca="false">IF($S140="","",IF(LEFT($S140,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S140="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S140="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S140="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S140="","",IF(LEFT($S140,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S140="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S140="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S140="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U140" s="19" t="str">
@@ -10247,7 +10247,7 @@
         <v/>
       </c>
       <c r="T141" s="18" t="str">
-        <f aca="false">IF($S141="","",IF(LEFT($S141,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S141="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S141="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S141="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S141="","",IF(LEFT($S141,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S141="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S141="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S141="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U141" s="19" t="str">
@@ -10306,7 +10306,7 @@
         <v/>
       </c>
       <c r="T142" s="18" t="str">
-        <f aca="false">IF($S142="","",IF(LEFT($S142,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S142="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S142="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S142="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S142="","",IF(LEFT($S142,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S142="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S142="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S142="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U142" s="19" t="str">
@@ -10365,7 +10365,7 @@
         <v/>
       </c>
       <c r="T143" s="18" t="str">
-        <f aca="false">IF($S143="","",IF(LEFT($S143,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S143="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S143="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S143="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S143="","",IF(LEFT($S143,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S143="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S143="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S143="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U143" s="19" t="str">
@@ -10424,7 +10424,7 @@
         <v/>
       </c>
       <c r="T144" s="18" t="str">
-        <f aca="false">IF($S144="","",IF(LEFT($S144,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S144="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S144="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S144="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S144="","",IF(LEFT($S144,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S144="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S144="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S144="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U144" s="19" t="str">
@@ -10483,7 +10483,7 @@
         <v/>
       </c>
       <c r="T145" s="18" t="str">
-        <f aca="false">IF($S145="","",IF(LEFT($S145,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S145="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S145="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S145="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S145="","",IF(LEFT($S145,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S145="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S145="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S145="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U145" s="19" t="str">
@@ -10542,7 +10542,7 @@
         <v/>
       </c>
       <c r="T146" s="18" t="str">
-        <f aca="false">IF($S146="","",IF(LEFT($S146,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S146="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S146="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S146="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S146="","",IF(LEFT($S146,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S146="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S146="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S146="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U146" s="19" t="str">
@@ -10601,7 +10601,7 @@
         <v/>
       </c>
       <c r="T147" s="18" t="str">
-        <f aca="false">IF($S147="","",IF(LEFT($S147,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S147="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S147="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S147="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S147="","",IF(LEFT($S147,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S147="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S147="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S147="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U147" s="19" t="str">
@@ -10660,7 +10660,7 @@
         <v/>
       </c>
       <c r="T148" s="18" t="str">
-        <f aca="false">IF($S148="","",IF(LEFT($S148,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S148="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S148="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S148="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S148="","",IF(LEFT($S148,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S148="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S148="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S148="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U148" s="19" t="str">
@@ -10719,7 +10719,7 @@
         <v/>
       </c>
       <c r="T149" s="18" t="str">
-        <f aca="false">IF($S149="","",IF(LEFT($S149,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S149="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S149="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S149="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S149="","",IF(LEFT($S149,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S149="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S149="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S149="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U149" s="19" t="str">
@@ -10778,7 +10778,7 @@
         <v/>
       </c>
       <c r="T150" s="18" t="str">
-        <f aca="false">IF($S150="","",IF(LEFT($S150,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S150="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S150="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S150="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S150="","",IF(LEFT($S150,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S150="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S150="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S150="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U150" s="19" t="str">
@@ -10837,7 +10837,7 @@
         <v/>
       </c>
       <c r="T151" s="18" t="str">
-        <f aca="false">IF($S151="","",IF(LEFT($S151,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S151="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S151="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S151="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S151="","",IF(LEFT($S151,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S151="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S151="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S151="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U151" s="19" t="str">
@@ -10896,7 +10896,7 @@
         <v/>
       </c>
       <c r="T152" s="18" t="str">
-        <f aca="false">IF($S152="","",IF(LEFT($S152,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S152="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S152="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S152="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S152="","",IF(LEFT($S152,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S152="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S152="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S152="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U152" s="19" t="str">
@@ -10955,7 +10955,7 @@
         <v/>
       </c>
       <c r="T153" s="18" t="str">
-        <f aca="false">IF($S153="","",IF(LEFT($S153,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S153="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S153="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S153="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S153="","",IF(LEFT($S153,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S153="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S153="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S153="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U153" s="19" t="str">
@@ -11014,7 +11014,7 @@
         <v/>
       </c>
       <c r="T154" s="18" t="str">
-        <f aca="false">IF($S154="","",IF(LEFT($S154,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S154="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S154="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S154="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <f aca="false">IF($S154="","",IF(LEFT($S154,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S154="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S154="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S154="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
         <v/>
       </c>
       <c r="U154" s="19" t="str">
@@ -14105,7 +14105,7 @@
       </c>
       <c r="C25" s="39" t="str">
         <f aca="false">T40</f>
-        <v>Pursue — trial + fast programme: 5% lifts read in 2–3 weeks</v>
+        <v>Pursue — trial + fast program: 5% lifts read in 2–3 weeks</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14197,8 +14197,8 @@
         <v>Tier 1</v>
       </c>
       <c r="T40" s="49" t="str">
-        <f aca="false">IF($S40="","",IF(LEFT($S40,6)="Tier 1","Pursue — trial + fast programme: 5% lifts read in 2–3 weeks",IF($S40="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S40="Tier 3","Deprioritise — only exceptional (20%) changes read in 3 weeks",IF($S40="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
-        <v>Pursue — trial + fast programme: 5% lifts read in 2–3 weeks</v>
+        <f aca="false">IF($S40="","",IF(LEFT($S40,6)="Tier 1","Pursue — trial + fast program: 5% lifts read in 2–3 weeks",IF($S40="Tier 2","Qualify — bold tests only (10%+ lifts); funnel-wide, 3-week reads",IF($S40="Tier 3","Deprioritize — only exceptional (20%) changes read in 3 weeks",IF($S40="Not a fit","Do not trial A/B — purchase tests cannot read in 3 weeks","Trial only if tests are scored on CTA clicks / leads, not purchases")))))</f>
+        <v>Pursue — trial + fast program: 5% lifts read in 2–3 weeks</v>
       </c>
       <c r="U40" s="50" t="n">
         <f aca="false">IF($L40="","",$L40*Assumptions!$C$17*$K40*12/1000000)</f>

</xml_diff>